<commit_message>
Reports Yml file configured
</commit_message>
<xml_diff>
--- a/testdata/login.xlsx
+++ b/testdata/login.xlsx
@@ -440,16 +440,16 @@
         <v>Pass@1234</v>
       </c>
       <c r="D2" t="str">
-        <v>Passed</v>
+        <v>Failed</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-09T08:45:22.788Z</v>
+        <v>2026-07-09T08:59:32.721Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-07-09T08:45:36.355Z</v>
+        <v>2026-07-09T08:59:38.571Z</v>
       </c>
       <c r="G2" t="str">
-        <v>13.57</v>
+        <v>5.85</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -466,16 +466,16 @@
         <v>Pass@123</v>
       </c>
       <c r="D3" t="str">
-        <v>Passed</v>
+        <v>Failed</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-07-09T08:45:22.910Z</v>
+        <v>2026-07-09T08:59:32.879Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-07-09T08:45:32.979Z</v>
+        <v>2026-07-09T08:59:38.391Z</v>
       </c>
       <c r="G3" t="str">
-        <v>10.07</v>
+        <v>5.51</v>
       </c>
       <c r="H3" t="str">
         <v/>

</xml_diff>